<commit_message>
Add alternate contact fields for pickup and delivery in shipment forms and templates
- Introduced fields for alternate contact person and number in the shipment creation and detail pages.
- Updated the shipment template to include alternate contact information.
- Adjusted related interfaces and state management to accommodate new fields.
</commit_message>
<xml_diff>
--- a/public/templates/fetcher-bulk-shipments-template.xlsx
+++ b/public/templates/fetcher-bulk-shipments-template.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:X1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -499,19 +499,23 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="26" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="34" customWidth="1" min="20" max="20"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="28" customWidth="1" min="18" max="18"/>
+    <col width="26" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="34" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -550,67 +554,87 @@
           <t>PICK UP CONTACT EMAIL</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>PICK UP ALTERNATE CONTACT PERSON</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>PICK UP ALTERNATE CONTACT NO</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>NO OF PIECES</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>WEIGHT (IN KG)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>DIMENSIONS (IN CM)</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>DELIVERY ADDRESS</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>DELIVERY PINCODE/ZIP CODE</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>DELIVERY CONTACT NO</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>DELIVERY CONTACT PERSON</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>DELIVERY CONTACT EMAIL</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>DELIVERY ALTERNATE CONTACT PERSON</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>DELIVERY ALTERNATE CONTACT NO</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>SHIPMENT TYPE</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>MODE</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>SHIPMENT CATAGORY</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>IS THIS A DG SHIPMENT?</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>ADDITIONAL INFORMATION</t>
         </is>
@@ -621,22 +645,22 @@
     <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Domestic, International" type="list" errorStyle="stop">
       <formula1>"Domestic,International"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
+    <dataValidation sqref="J2:J501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
+    <dataValidation sqref="K2:K501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Commercial, Non-Commercial" type="list" errorStyle="stop">
+    <dataValidation sqref="T2:T501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Commercial, Non-Commercial" type="list" errorStyle="stop">
       <formula1>"Commercial,Non-Commercial"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Express, Air, Surface, Eco-Ground" type="list" errorStyle="stop">
+    <dataValidation sqref="U2:U501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Express, Air, Surface, Eco-Ground" type="list" errorStyle="stop">
       <formula1>"Express,Air,Surface,Eco-Ground"</formula1>
     </dataValidation>
-    <dataValidation sqref="R2:R501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Doc, Non-Doc" type="list" errorStyle="stop">
+    <dataValidation sqref="V2:V501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Doc, Non-Doc" type="list" errorStyle="stop">
       <formula1>"Doc,Non-Doc"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Yes, No" type="list" errorStyle="stop">
+    <dataValidation sqref="W2:W501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Yes, No" type="list" errorStyle="stop">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -650,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -878,58 +902,58 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>NO OF PIECES</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>PICK UP ALTERNATE CONTACT PERSON</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Whole number, at least 1</t>
+          <t>Backup contact name at pickup (optional)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>WEIGHT (IN KG)</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>PICK UP ALTERNATE CONTACT NO</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Number greater than 0</t>
+          <t>Backup contact phone at pickup (optional)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>DIMENSIONS (IN CM)</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
+          <t>NO OF PIECES</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>e.g. 30x20x15 (optional)</t>
+          <t>Whole number, at least 1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY ADDRESS</t>
+          <t>WEIGHT (IN KG)</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
@@ -939,31 +963,31 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Full delivery address</t>
+          <t>Number greater than 0</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY PINCODE/ZIP CODE</t>
-        </is>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>DIMENSIONS (IN CM)</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Delivery pincode / ZIP code</t>
+          <t>e.g. 30x20x15 (optional)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY CONTACT NO</t>
+          <t>DELIVERY ADDRESS</t>
         </is>
       </c>
       <c r="B27" s="10" t="inlineStr">
@@ -973,99 +997,99 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Contact phone at delivery</t>
+          <t>Full delivery address</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY CONTACT PERSON</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
+          <t>DELIVERY PINCODE/ZIP CODE</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Contact name at delivery (optional)</t>
+          <t>Delivery pincode / ZIP code</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY CONTACT EMAIL</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
+          <t>DELIVERY CONTACT NO</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Contact email at delivery (optional)</t>
+          <t>Contact phone at delivery</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>SHIPMENT TYPE</t>
-        </is>
-      </c>
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>DELIVERY CONTACT PERSON</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Dropdown: Commercial / Non-Commercial</t>
+          <t>Contact name at delivery (optional)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>MODE</t>
-        </is>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>DELIVERY CONTACT EMAIL</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Dropdown: Express / Air / Surface / Eco-Ground</t>
+          <t>Contact email at delivery (optional)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>SHIPMENT CATAGORY</t>
-        </is>
-      </c>
-      <c r="B32" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>DELIVERY ALTERNATE CONTACT PERSON</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Dropdown: Doc / Non-Doc</t>
+          <t>Backup contact name at delivery (optional)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>IS THIS A DG SHIPMENT?</t>
+          <t>DELIVERY ALTERNATE CONTACT NO</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -1075,38 +1099,106 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Dropdown: Yes / No (blank = No)</t>
+          <t>Backup contact phone at delivery (optional)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
+          <t>SHIPMENT TYPE</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Dropdown: Commercial / Non-Commercial</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>MODE</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Dropdown: Express / Air / Surface / Eco-Ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>SHIPMENT CATAGORY</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Dropdown: Doc / Non-Doc</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>IS THIS A DG SHIPMENT?</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Dropdown: Yes / No (blank = No)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
           <t>ADDITIONAL INFORMATION</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>Any extra notes (optional)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>Example row</t>
         </is>
       </c>
-      <c r="B36" s="6" t="n"/>
-      <c r="C36" s="6" t="n"/>
-    </row>
-    <row r="37" ht="60" customHeight="1">
-      <c r="A37" s="7" t="inlineStr">
+      <c r="B40" s="6" t="n"/>
+      <c r="C40" s="6" t="n"/>
+    </row>
+    <row r="41" ht="60" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
         <is>
           <t>REF=ORD-1001 | SCOPE=Domestic | PICK UP ADDRESS=12 MG Road, Bengaluru 560001 | PICK UP PINCODE/ZIP CODE=560001 | PICK UP CONTACT NO=9876543210 | NO OF PIECES=2 | WEIGHT (IN KG)=5.5 | DELIVERY ADDRESS=4 Park Street, Kolkata 700016 | DELIVERY PINCODE/ZIP CODE=700016 | DELIVERY CONTACT NO=9123456780 | SHIPMENT TYPE=Commercial | MODE=Express | SHIPMENT CATAGORY=Non-Doc | IS THIS A DG SHIPMENT?=No</t>
         </is>
@@ -1115,9 +1207,9 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A41:C41"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A37:C37"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A9:C9"/>

</xml_diff>

<commit_message>
Enhance bulk shipment template to support multiple parcels
- Updated the bulk shipment template to accommodate up to 5 parcels, including fields for pieces, weight, and dimensions for each parcel.
- Refactored the generation script to dynamically create column headers and validation rules for the new parcel structure.
- Improved user instructions to clarify how to fill out parcel information in the template.
</commit_message>
<xml_diff>
--- a/public/templates/fetcher-bulk-shipments-template.xlsx
+++ b/public/templates/fetcher-bulk-shipments-template.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:AJ1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -501,21 +501,33 @@
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
-    <col width="28" customWidth="1" min="18" max="18"/>
-    <col width="26" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="22" customWidth="1" min="23" max="23"/>
-    <col width="34" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="17" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="40" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="26" customWidth="1" min="29" max="29"/>
+    <col width="28" customWidth="1" min="30" max="30"/>
+    <col width="26" customWidth="1" min="31" max="31"/>
+    <col width="18" customWidth="1" min="32" max="32"/>
+    <col width="16" customWidth="1" min="33" max="33"/>
+    <col width="18" customWidth="1" min="34" max="34"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
+    <col width="34" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -566,82 +578,142 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>NO OF PIECES</t>
+          <t>PARCEL 1 NO OF PIECES</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>WEIGHT (IN KG)</t>
+          <t>PARCEL 1 WEIGHT (IN KG)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>DIMENSIONS (IN CM)</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
+          <t>PARCEL 1 DIMENSIONS (IN CM)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>PARCEL 2 NO OF PIECES</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>PARCEL 2 WEIGHT (IN KG)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>PARCEL 2 DIMENSIONS (IN CM)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>PARCEL 3 NO OF PIECES</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>PARCEL 3 WEIGHT (IN KG)</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>PARCEL 3 DIMENSIONS (IN CM)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>PARCEL 4 NO OF PIECES</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>PARCEL 4 WEIGHT (IN KG)</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>PARCEL 4 DIMENSIONS (IN CM)</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>PARCEL 5 NO OF PIECES</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>PARCEL 5 WEIGHT (IN KG)</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>PARCEL 5 DIMENSIONS (IN CM)</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>DELIVERY ADDRESS</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>DELIVERY PINCODE/ZIP CODE</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>DELIVERY CONTACT NO</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>DELIVERY CONTACT PERSON</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>DELIVERY CONTACT EMAIL</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>DELIVERY ALTERNATE CONTACT PERSON</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>DELIVERY ALTERNATE CONTACT NO</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="AF1" s="2" t="inlineStr">
         <is>
           <t>SHIPMENT TYPE</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="AG1" s="2" t="inlineStr">
         <is>
           <t>MODE</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="AH1" s="2" t="inlineStr">
         <is>
           <t>SHIPMENT CATAGORY</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>IS THIS A DG SHIPMENT?</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>ADDITIONAL INFORMATION</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="7">
+  <dataValidations count="15">
     <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Domestic, International" type="list" errorStyle="stop">
       <formula1>"Domestic,International"</formula1>
     </dataValidation>
@@ -651,16 +723,40 @@
     <dataValidation sqref="K2:K501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="T2:T501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Commercial, Non-Commercial" type="list" errorStyle="stop">
+    <dataValidation sqref="M2:M501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="P2:P501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation sqref="Q2:Q501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="S2:S501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation sqref="T2:T501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="V2:V501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation sqref="W2:W501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF2:AF501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Commercial, Non-Commercial" type="list" errorStyle="stop">
       <formula1>"Commercial,Non-Commercial"</formula1>
     </dataValidation>
-    <dataValidation sqref="U2:U501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Express, Air, Surface, Eco-Ground" type="list" errorStyle="stop">
+    <dataValidation sqref="AG2:AG501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Express, Air, Surface, Eco-Ground" type="list" errorStyle="stop">
       <formula1>"Express,Air,Surface,Eco-Ground"</formula1>
     </dataValidation>
-    <dataValidation sqref="V2:V501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Doc, Non-Doc" type="list" errorStyle="stop">
+    <dataValidation sqref="AH2:AH501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Doc, Non-Doc" type="list" errorStyle="stop">
       <formula1>"Doc,Non-Doc"</formula1>
     </dataValidation>
-    <dataValidation sqref="W2:W501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Yes, No" type="list" errorStyle="stop">
+    <dataValidation sqref="AI2:AI501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Yes, No" type="list" errorStyle="stop">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -674,7 +770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -743,81 +839,71 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>•  Leave AWB, Client ID, Status, Billing, etc. out — they are assigned automatically by Fetcher / ops.</t>
+          <t>•  A shipment can have up to 5 parcels: fill PARCEL 1, then add PARCEL 2–5 only if there are more boxes.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
+          <t>•  Leave AWB, Client ID, Status, Billing, etc. out — they are assigned automatically by Fetcher / ops.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t>•  REF is your own optional reference; we echo it back in the results so you can match any errors to your rows.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Columns</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Allowed values / format</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>REF</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Your own reference (optional) — echoed back in the results so you can match errors to rows.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>SCOPE</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>REF</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Dropdown: Domestic / International</t>
+          <t>Your own reference (optional) — echoed back in the results so you can match errors to rows.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>PICK UP ADDRESS</t>
+          <t>SCOPE</t>
         </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
@@ -827,14 +913,14 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Full pickup address</t>
+          <t>Dropdown: Domestic / International</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>PICK UP PINCODE/ZIP CODE</t>
+          <t>PICK UP ADDRESS</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
@@ -844,65 +930,65 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Pickup pincode / ZIP code</t>
+          <t>Full pickup address</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>PICK UP CONTACT PERSON</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
+          <t>PICK UP PINCODE/ZIP CODE</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Contact name at pickup (optional)</t>
+          <t>Pickup pincode / ZIP code</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>PICK UP CONTACT NO</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>PICK UP CONTACT PERSON</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Contact phone at pickup</t>
+          <t>Contact name at pickup (optional)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>PICK UP CONTACT EMAIL</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
+          <t>PICK UP CONTACT NO</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Contact email at pickup (optional)</t>
+          <t>Contact phone at pickup</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>PICK UP ALTERNATE CONTACT PERSON</t>
+          <t>PICK UP CONTACT EMAIL</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -912,14 +998,14 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Backup contact name at pickup (optional)</t>
+          <t>Contact email at pickup (optional)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>PICK UP ALTERNATE CONTACT NO</t>
+          <t>PICK UP ALTERNATE CONTACT PERSON</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -929,31 +1015,31 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Backup contact phone at pickup (optional)</t>
+          <t>Backup contact name at pickup (optional)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>NO OF PIECES</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>PICK UP ALTERNATE CONTACT NO</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Whole number, at least 1</t>
+          <t>Backup contact phone at pickup (optional)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>WEIGHT (IN KG)</t>
+          <t>PARCEL 1 NO OF PIECES</t>
         </is>
       </c>
       <c r="B25" s="10" t="inlineStr">
@@ -963,82 +1049,82 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Number greater than 0</t>
+          <t>Whole number, at least 1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>DIMENSIONS (IN CM)</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
+          <t>PARCEL 1 WEIGHT (IN KG)</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>e.g. 30x20x15 (optional)</t>
+          <t>Number greater than 0</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY ADDRESS</t>
-        </is>
-      </c>
-      <c r="B27" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>PARCEL 1 DIMENSIONS (IN CM)</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Full delivery address</t>
+          <t>e.g. 30x20x15 (optional)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY PINCODE/ZIP CODE</t>
-        </is>
-      </c>
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>PARCEL 2 NO OF PIECES</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Delivery pincode / ZIP code</t>
+          <t>Whole number, at least 1 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY CONTACT NO</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>PARCEL 2 WEIGHT (IN KG)</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Contact phone at delivery</t>
+          <t>Number greater than 0 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY CONTACT PERSON</t>
+          <t>PARCEL 2 DIMENSIONS (IN CM)</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -1048,14 +1134,14 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Contact name at delivery (optional)</t>
+          <t>e.g. 30x20x15 (optional)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY CONTACT EMAIL</t>
+          <t>PARCEL 3 NO OF PIECES</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -1065,14 +1151,14 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Contact email at delivery (optional)</t>
+          <t>Whole number, at least 1 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY ALTERNATE CONTACT PERSON</t>
+          <t>PARCEL 3 WEIGHT (IN KG)</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -1082,14 +1168,14 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Backup contact name at delivery (optional)</t>
+          <t>Number greater than 0 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY ALTERNATE CONTACT NO</t>
+          <t>PARCEL 3 DIMENSIONS (IN CM)</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -1099,65 +1185,65 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Backup contact phone at delivery (optional)</t>
+          <t>e.g. 30x20x15 (optional)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>SHIPMENT TYPE</t>
-        </is>
-      </c>
-      <c r="B34" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>PARCEL 4 NO OF PIECES</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Dropdown: Commercial / Non-Commercial</t>
+          <t>Whole number, at least 1 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>MODE</t>
-        </is>
-      </c>
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>PARCEL 4 WEIGHT (IN KG)</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Dropdown: Express / Air / Surface / Eco-Ground</t>
+          <t>Number greater than 0 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>SHIPMENT CATAGORY</t>
-        </is>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>PARCEL 4 DIMENSIONS (IN CM)</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Dropdown: Doc / Non-Doc</t>
+          <t>e.g. 30x20x15 (optional)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>IS THIS A DG SHIPMENT?</t>
+          <t>PARCEL 5 NO OF PIECES</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -1167,53 +1253,275 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Dropdown: Yes / No (blank = No)</t>
+          <t>Whole number, at least 1 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
+          <t>PARCEL 5 WEIGHT (IN KG)</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Number greater than 0 — only if this parcel is used</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>PARCEL 5 DIMENSIONS (IN CM)</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>e.g. 30x20x15 (optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>DELIVERY ADDRESS</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Full delivery address</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>DELIVERY PINCODE/ZIP CODE</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Delivery pincode / ZIP code</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>DELIVERY CONTACT NO</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Contact phone at delivery</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>DELIVERY CONTACT PERSON</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Contact name at delivery (optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="9" t="inlineStr">
+        <is>
+          <t>DELIVERY CONTACT EMAIL</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Contact email at delivery (optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="9" t="inlineStr">
+        <is>
+          <t>DELIVERY ALTERNATE CONTACT PERSON</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Backup contact name at delivery (optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>DELIVERY ALTERNATE CONTACT NO</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Backup contact phone at delivery (optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="9" t="inlineStr">
+        <is>
+          <t>SHIPMENT TYPE</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Dropdown: Commercial / Non-Commercial</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>MODE</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Dropdown: Express / Air / Surface / Eco-Ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>SHIPMENT CATAGORY</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Dropdown: Doc / Non-Doc</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>IS THIS A DG SHIPMENT?</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Dropdown: Yes / No (blank = No)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
           <t>ADDITIONAL INFORMATION</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
         <is>
           <t>Any extra notes (optional)</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>Example row</t>
         </is>
       </c>
-      <c r="B40" s="6" t="n"/>
-      <c r="C40" s="6" t="n"/>
-    </row>
-    <row r="41" ht="60" customHeight="1">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>REF=ORD-1001 | SCOPE=Domestic | PICK UP ADDRESS=12 MG Road, Bengaluru 560001 | PICK UP PINCODE/ZIP CODE=560001 | PICK UP CONTACT NO=9876543210 | NO OF PIECES=2 | WEIGHT (IN KG)=5.5 | DELIVERY ADDRESS=4 Park Street, Kolkata 700016 | DELIVERY PINCODE/ZIP CODE=700016 | DELIVERY CONTACT NO=9123456780 | SHIPMENT TYPE=Commercial | MODE=Express | SHIPMENT CATAGORY=Non-Doc | IS THIS A DG SHIPMENT?=No</t>
+      <c r="B53" s="6" t="n"/>
+      <c r="C53" s="6" t="n"/>
+    </row>
+    <row r="54" ht="60" customHeight="1">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>REF=ORD-1001 | SCOPE=Domestic | PICK UP ADDRESS=12 MG Road, Bengaluru 560001 | PICK UP PINCODE/ZIP CODE=560001 | PICK UP CONTACT NO=9876543210 | PARCEL 1 NO OF PIECES=2 | PARCEL 1 WEIGHT (IN KG)=5.5 | PARCEL 1 DIMENSIONS (IN CM)=30x20x15 | PARCEL 2 NO OF PIECES=1 | PARCEL 2 WEIGHT (IN KG)=3 | DELIVERY ADDRESS=4 Park Street, Kolkata 700016 | DELIVERY PINCODE/ZIP CODE=700016 | DELIVERY CONTACT NO=9123456780 | SHIPMENT TYPE=Commercial | MODE=Express | SHIPMENT CATAGORY=Non-Doc | IS THIS A DG SHIPMENT?=No</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A41:C41"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A12:C12"/>
     <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A54:C54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add City and State address fields with state dropdown and pincode auto-fill
</commit_message>
<xml_diff>
--- a/public/templates/fetcher-bulk-shipments-template.xlsx
+++ b/public/templates/fetcher-bulk-shipments-template.xlsx
@@ -489,45 +489,49 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ1"/>
+  <dimension ref="A1:AN1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="17" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="17" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="17" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
-    <col width="40" customWidth="1" min="25" max="25"/>
-    <col width="20" customWidth="1" min="26" max="26"/>
-    <col width="18" customWidth="1" min="27" max="27"/>
-    <col width="22" customWidth="1" min="28" max="28"/>
-    <col width="26" customWidth="1" min="29" max="29"/>
-    <col width="28" customWidth="1" min="30" max="30"/>
-    <col width="26" customWidth="1" min="31" max="31"/>
-    <col width="18" customWidth="1" min="32" max="32"/>
-    <col width="16" customWidth="1" min="33" max="33"/>
-    <col width="18" customWidth="1" min="34" max="34"/>
-    <col width="22" customWidth="1" min="35" max="35"/>
-    <col width="34" customWidth="1" min="36" max="36"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="17" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="17" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="16" customWidth="1" min="24" max="24"/>
+    <col width="17" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="40" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="28" max="28"/>
+    <col width="20" customWidth="1" min="29" max="29"/>
+    <col width="20" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="22" customWidth="1" min="32" max="32"/>
+    <col width="26" customWidth="1" min="33" max="33"/>
+    <col width="28" customWidth="1" min="34" max="34"/>
+    <col width="26" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
+    <col width="16" customWidth="1" min="37" max="37"/>
+    <col width="18" customWidth="1" min="38" max="38"/>
+    <col width="22" customWidth="1" min="39" max="39"/>
+    <col width="34" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -548,165 +552,185 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
+          <t>PICK UP CITY</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>PICK UP STATE</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
           <t>PICK UP PINCODE/ZIP CODE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>PICK UP CONTACT PERSON</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>PICK UP CONTACT NO</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>PICK UP CONTACT EMAIL</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>PICK UP ALTERNATE CONTACT PERSON</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>PICK UP ALTERNATE CONTACT NO</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>PARCEL 1 NO OF PIECES</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>PARCEL 1 WEIGHT (IN KG)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>PARCEL 1 DIMENSIONS (IN CM)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>PARCEL 2 NO OF PIECES</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>PARCEL 2 WEIGHT (IN KG)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>PARCEL 2 DIMENSIONS (IN CM)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>PARCEL 3 NO OF PIECES</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>PARCEL 3 WEIGHT (IN KG)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>PARCEL 3 DIMENSIONS (IN CM)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>PARCEL 4 NO OF PIECES</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>PARCEL 4 WEIGHT (IN KG)</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>PARCEL 4 DIMENSIONS (IN CM)</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>PARCEL 5 NO OF PIECES</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>PARCEL 5 WEIGHT (IN KG)</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>PARCEL 5 DIMENSIONS (IN CM)</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>DELIVERY ADDRESS</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>DELIVERY CITY</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
+        <is>
+          <t>DELIVERY STATE</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>DELIVERY PINCODE/ZIP CODE</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AE1" s="2" t="inlineStr">
         <is>
           <t>DELIVERY CONTACT NO</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>DELIVERY CONTACT PERSON</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>DELIVERY CONTACT EMAIL</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>DELIVERY ALTERNATE CONTACT PERSON</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>DELIVERY ALTERNATE CONTACT NO</t>
         </is>
       </c>
-      <c r="AF1" s="2" t="inlineStr">
+      <c r="AJ1" s="2" t="inlineStr">
         <is>
           <t>SHIPMENT TYPE</t>
         </is>
       </c>
-      <c r="AG1" s="2" t="inlineStr">
+      <c r="AK1" s="2" t="inlineStr">
         <is>
           <t>MODE</t>
         </is>
       </c>
-      <c r="AH1" s="2" t="inlineStr">
+      <c r="AL1" s="2" t="inlineStr">
         <is>
           <t>SHIPMENT CATAGORY</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>IS THIS A DG SHIPMENT?</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>ADDITIONAL INFORMATION</t>
         </is>
@@ -717,46 +741,46 @@
     <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Domestic, International" type="list" errorStyle="stop">
       <formula1>"Domestic,International"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
+    <dataValidation sqref="L2:L501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
+    <dataValidation sqref="M2:M501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
+    <dataValidation sqref="O2:O501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
+    <dataValidation sqref="P2:P501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
+    <dataValidation sqref="R2:R501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
+    <dataValidation sqref="S2:S501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
+    <dataValidation sqref="U2:U501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation sqref="T2:T501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
+    <dataValidation sqref="V2:V501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="V2:V501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
+    <dataValidation sqref="X2:X501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid number" error="No. of pieces must be a whole number of at least 1." type="whole" errorStyle="stop" operator="greaterThanOrEqual">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation sqref="W2:W501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
+    <dataValidation sqref="Y2:Y501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid weight" error="Weight (kg) must be a number greater than 0." type="decimal" errorStyle="stop" operator="greaterThan">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation sqref="AF2:AF501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Commercial, Non-Commercial" type="list" errorStyle="stop">
+    <dataValidation sqref="AJ2:AJ501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Commercial, Non-Commercial" type="list" errorStyle="stop">
       <formula1>"Commercial,Non-Commercial"</formula1>
     </dataValidation>
-    <dataValidation sqref="AG2:AG501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Express, Air, Surface, Eco-Ground" type="list" errorStyle="stop">
+    <dataValidation sqref="AK2:AK501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Express, Air, Surface, Eco-Ground" type="list" errorStyle="stop">
       <formula1>"Express,Air,Surface,Eco-Ground"</formula1>
     </dataValidation>
-    <dataValidation sqref="AH2:AH501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Doc, Non-Doc" type="list" errorStyle="stop">
+    <dataValidation sqref="AL2:AL501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Doc, Non-Doc" type="list" errorStyle="stop">
       <formula1>"Doc,Non-Doc"</formula1>
     </dataValidation>
-    <dataValidation sqref="AI2:AI501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Yes, No" type="list" errorStyle="stop">
+    <dataValidation sqref="AM2:AM501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Choose one of: Yes, No" type="list" errorStyle="stop">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -770,7 +794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -937,7 +961,7 @@
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>PICK UP PINCODE/ZIP CODE</t>
+          <t>PICK UP CITY</t>
         </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
@@ -947,31 +971,31 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Pickup pincode / ZIP code</t>
+          <t>Pickup city</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>PICK UP CONTACT PERSON</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
+          <t>PICK UP STATE</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Contact name at pickup (optional)</t>
+          <t>Pickup state — required for Domestic; use the full state name (e.g. Karnataka)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>PICK UP CONTACT NO</t>
+          <t>PICK UP PINCODE/ZIP CODE</t>
         </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
@@ -981,14 +1005,14 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Contact phone at pickup</t>
+          <t>Pickup pincode / ZIP code</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>PICK UP CONTACT EMAIL</t>
+          <t>PICK UP CONTACT PERSON</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -998,31 +1022,31 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Contact email at pickup (optional)</t>
+          <t>Contact name at pickup (optional)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>PICK UP ALTERNATE CONTACT PERSON</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
+          <t>PICK UP CONTACT NO</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Backup contact name at pickup (optional)</t>
+          <t>Contact phone at pickup</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>PICK UP ALTERNATE CONTACT NO</t>
+          <t>PICK UP CONTACT EMAIL</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -1032,82 +1056,82 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Backup contact phone at pickup (optional)</t>
+          <t>Contact email at pickup (optional)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 1 NO OF PIECES</t>
-        </is>
-      </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>PICK UP ALTERNATE CONTACT PERSON</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Whole number, at least 1</t>
+          <t>Backup contact name at pickup (optional)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 1 WEIGHT (IN KG)</t>
-        </is>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>PICK UP ALTERNATE CONTACT NO</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Number greater than 0</t>
+          <t>Backup contact phone at pickup (optional)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 1 DIMENSIONS (IN CM)</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
+          <t>PARCEL 1 NO OF PIECES</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>e.g. 30x20x15 (optional)</t>
+          <t>Whole number, at least 1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 2 NO OF PIECES</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
+          <t>PARCEL 1 WEIGHT (IN KG)</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Whole number, at least 1 — only if this parcel is used</t>
+          <t>Number greater than 0</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 2 WEIGHT (IN KG)</t>
+          <t>PARCEL 1 DIMENSIONS (IN CM)</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
@@ -1117,14 +1141,14 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Number greater than 0 — only if this parcel is used</t>
+          <t>e.g. 30x20x15 (optional)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 2 DIMENSIONS (IN CM)</t>
+          <t>PARCEL 2 NO OF PIECES</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
@@ -1134,14 +1158,14 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>e.g. 30x20x15 (optional)</t>
+          <t>Whole number, at least 1 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 3 NO OF PIECES</t>
+          <t>PARCEL 2 WEIGHT (IN KG)</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -1151,14 +1175,14 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Whole number, at least 1 — only if this parcel is used</t>
+          <t>Number greater than 0 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 3 WEIGHT (IN KG)</t>
+          <t>PARCEL 2 DIMENSIONS (IN CM)</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
@@ -1168,14 +1192,14 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Number greater than 0 — only if this parcel is used</t>
+          <t>e.g. 30x20x15 (optional)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 3 DIMENSIONS (IN CM)</t>
+          <t>PARCEL 3 NO OF PIECES</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
@@ -1185,14 +1209,14 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>e.g. 30x20x15 (optional)</t>
+          <t>Whole number, at least 1 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 4 NO OF PIECES</t>
+          <t>PARCEL 3 WEIGHT (IN KG)</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
@@ -1202,14 +1226,14 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Whole number, at least 1 — only if this parcel is used</t>
+          <t>Number greater than 0 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 4 WEIGHT (IN KG)</t>
+          <t>PARCEL 3 DIMENSIONS (IN CM)</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
@@ -1219,14 +1243,14 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Number greater than 0 — only if this parcel is used</t>
+          <t>e.g. 30x20x15 (optional)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 4 DIMENSIONS (IN CM)</t>
+          <t>PARCEL 4 NO OF PIECES</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
@@ -1236,14 +1260,14 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>e.g. 30x20x15 (optional)</t>
+          <t>Whole number, at least 1 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 5 NO OF PIECES</t>
+          <t>PARCEL 4 WEIGHT (IN KG)</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
@@ -1253,14 +1277,14 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Whole number, at least 1 — only if this parcel is used</t>
+          <t>Number greater than 0 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 5 WEIGHT (IN KG)</t>
+          <t>PARCEL 4 DIMENSIONS (IN CM)</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -1270,14 +1294,14 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Number greater than 0 — only if this parcel is used</t>
+          <t>e.g. 30x20x15 (optional)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>PARCEL 5 DIMENSIONS (IN CM)</t>
+          <t>PARCEL 5 NO OF PIECES</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
@@ -1287,48 +1311,48 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>e.g. 30x20x15 (optional)</t>
+          <t>Whole number, at least 1 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY ADDRESS</t>
-        </is>
-      </c>
-      <c r="B40" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>PARCEL 5 WEIGHT (IN KG)</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Full delivery address</t>
+          <t>Number greater than 0 — only if this parcel is used</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY PINCODE/ZIP CODE</t>
-        </is>
-      </c>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>PARCEL 5 DIMENSIONS (IN CM)</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Delivery pincode / ZIP code</t>
+          <t>e.g. 30x20x15 (optional)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY CONTACT NO</t>
+          <t>DELIVERY ADDRESS</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
@@ -1338,133 +1362,133 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Contact phone at delivery</t>
+          <t>Full delivery address</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY CONTACT PERSON</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
+          <t>DELIVERY CITY</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Contact name at delivery (optional)</t>
+          <t>Delivery city</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY CONTACT EMAIL</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
+          <t>DELIVERY STATE</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Contact email at delivery (optional)</t>
+          <t>Delivery state — required for Domestic; use the full state name (e.g. West Bengal)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY ALTERNATE CONTACT PERSON</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
+          <t>DELIVERY PINCODE/ZIP CODE</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Backup contact name at delivery (optional)</t>
+          <t>Delivery pincode / ZIP code</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>DELIVERY ALTERNATE CONTACT NO</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
+          <t>DELIVERY CONTACT NO</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Backup contact phone at delivery (optional)</t>
+          <t>Contact phone at delivery</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>SHIPMENT TYPE</t>
-        </is>
-      </c>
-      <c r="B47" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>DELIVERY CONTACT PERSON</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Dropdown: Commercial / Non-Commercial</t>
+          <t>Contact name at delivery (optional)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>MODE</t>
-        </is>
-      </c>
-      <c r="B48" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>DELIVERY CONTACT EMAIL</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Dropdown: Express / Air / Surface / Eco-Ground</t>
+          <t>Contact email at delivery (optional)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>SHIPMENT CATAGORY</t>
-        </is>
-      </c>
-      <c r="B49" s="10" t="inlineStr">
-        <is>
-          <t>Required</t>
+          <t>DELIVERY ALTERNATE CONTACT PERSON</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Dropdown: Doc / Non-Doc</t>
+          <t>Backup contact name at delivery (optional)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>IS THIS A DG SHIPMENT?</t>
+          <t>DELIVERY ALTERNATE CONTACT NO</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
@@ -1474,40 +1498,108 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Dropdown: Yes / No (blank = No)</t>
+          <t>Backup contact phone at delivery (optional)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
+          <t>SHIPMENT TYPE</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Dropdown: Commercial / Non-Commercial</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>MODE</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Dropdown: Express / Air / Surface / Eco-Ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>SHIPMENT CATAGORY</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Dropdown: Doc / Non-Doc</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="9" t="inlineStr">
+        <is>
+          <t>IS THIS A DG SHIPMENT?</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Dropdown: Yes / No (blank = No)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="inlineStr">
+        <is>
           <t>ADDITIONAL INFORMATION</t>
         </is>
       </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
         <is>
           <t>Any extra notes (optional)</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>Example row</t>
         </is>
       </c>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="6" t="n"/>
-    </row>
-    <row r="54" ht="60" customHeight="1">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>REF=ORD-1001 | SCOPE=Domestic | PICK UP ADDRESS=12 MG Road, Bengaluru 560001 | PICK UP PINCODE/ZIP CODE=560001 | PICK UP CONTACT NO=9876543210 | PARCEL 1 NO OF PIECES=2 | PARCEL 1 WEIGHT (IN KG)=5.5 | PARCEL 1 DIMENSIONS (IN CM)=30x20x15 | PARCEL 2 NO OF PIECES=1 | PARCEL 2 WEIGHT (IN KG)=3 | DELIVERY ADDRESS=4 Park Street, Kolkata 700016 | DELIVERY PINCODE/ZIP CODE=700016 | DELIVERY CONTACT NO=9123456780 | SHIPMENT TYPE=Commercial | MODE=Express | SHIPMENT CATAGORY=Non-Doc | IS THIS A DG SHIPMENT?=No</t>
+      <c r="B57" s="6" t="n"/>
+      <c r="C57" s="6" t="n"/>
+    </row>
+    <row r="58" ht="60" customHeight="1">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>REF=ORD-1001 | SCOPE=Domestic | PICK UP ADDRESS=12 MG Road, Bengaluru 560001 | PICK UP CITY=Bengaluru | PICK UP STATE=Karnataka | PICK UP PINCODE/ZIP CODE=560001 | PICK UP CONTACT NO=9876543210 | PARCEL 1 NO OF PIECES=2 | PARCEL 1 WEIGHT (IN KG)=5.5 | PARCEL 1 DIMENSIONS (IN CM)=30x20x15 | PARCEL 2 NO OF PIECES=1 | PARCEL 2 WEIGHT (IN KG)=3 | DELIVERY ADDRESS=4 Park Street, Kolkata 700016 | DELIVERY CITY=Kolkata | DELIVERY STATE=West Bengal | DELIVERY PINCODE/ZIP CODE=700016 | DELIVERY CONTACT NO=9123456780 | SHIPMENT TYPE=Commercial | MODE=Express | SHIPMENT CATAGORY=Non-Doc | IS THIS A DG SHIPMENT?=No</t>
         </is>
       </c>
     </row>
@@ -1518,10 +1610,10 @@
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A58:C58"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A54:C54"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>